<commit_message>
Research report: describe Vietnam 2010/11 as a level shift, not a series break
USDA shows Vietnam at 17-19.5 M bags from 2006/07 to 2010/11, then 26.0 M
in 2011/12 (+34 %). Exports follow (+31 %), official Vietnamese statistics
(FAOSTAT) show +15 %. The report now says this, explains why the robusta
analysis starts in 2011/12, and states that Vietnam remains the largest
robusta producer by volume even though conilon drives more of the swings.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hsy3bDWLR2oyncbyTiqnwU
</commit_message>
<xml_diff>
--- a/coffee_stu/Recherche_STU_prix_cafe.xlsx
+++ b/coffee_stu/Recherche_STU_prix_cafe.xlsx
@@ -52,7 +52,7 @@
     <t>8_KC_DF : KC et DF au mois (même unité, c/lb), ratio KC/DF, corrélations de référence, statistiques du ratio, récoltes par espèce et ratio par campagne (graphique).</t>
   </si>
   <si>
-    <t>Après vérification : validation croisée sans 2023/24-2025/26 et réaction des stocks au prix (6_STU_prix), intervalles bootstrap (2_Chocs), crise année par année (3_Crise), tendances 2011/12-2025/26 sans la rupture de série du Vietnam en 2010/11 (2_Chocs, 4_Long_terme, 5_Production_prix).</t>
+    <t>Après vérification : validation croisée sans 2023/24-2025/26 et réaction des stocks au prix (6_STU_prix), intervalles bootstrap (2_Chocs), crise année par année (3_Crise), tendances 2011/12-2025/26 sans le saut de niveau du Vietnam entre 2010/11 et 2011/12 (2_Chocs, 4_Long_terme, 5_Production_prix).</t>
   </si>
   <si>
     <t>Pièges : consommation UE apparente (miroir des stocks) ; UE regroupée avec le Royaume-Uni (passage UE-28 -&gt; UE-27 en 2016/17) ; stocks américains figés à 5,7 M sacs depuis 2022/23 ; bosse des stocks indonésiens 2017-2021 ; exportations mondiales &gt; importations de 1 à 13 M sacs par an. 16 campagnes : ordres de grandeur, pas des preuves.</t>
@@ -274,7 +274,7 @@
     <t>Arabica brésilien premier dans 90 % des 4000 tirages bootstrap ; P(conilon &gt; Vietnam) = 0.71.</t>
   </si>
   <si>
-    <t>Fenêtre 2011/12-2025/26 (sans la rupture de série du Vietnam en 2010/11) : taille des écarts à la tendance</t>
+    <t>Fenêtre 2011/12-2025/26 (sans le saut de niveau du Vietnam entre 2010/11 et 2011/12) : taille des écarts à la tendance</t>
   </si>
   <si>
     <t>Origine</t>
@@ -472,7 +472,7 @@
     <t>Tendance 2011/12-2025/26 (M sacs par an)</t>
   </si>
   <si>
-    <t>Les bornes 2010/11 et 2025/26 sont trompeuses pour le Brésil arabica (année haute puis année basse) et le Vietnam (2010/11 = rupture de série, 19,4 M sacs) : préférer la tendance 2011/12-2025/26.</t>
+    <t>Les bornes 2010/11 et 2025/26 sont trompeuses pour le Brésil arabica (année haute puis année basse) et le Vietnam (saut de niveau : 19,4 M sacs en 2010/11, 26,0 M en 2011/12) : préférer la tendance 2011/12-2025/26.</t>
   </si>
   <si>
     <t>Production par origine et prix : corrélations des variations annuelles (n = 15)</t>
@@ -577,7 +577,7 @@
     <t>Les corrélations à ±1 mois (+0,19 et +0,14) ont la taille que produit le seul calcul de moyennes mensuelles (environ 0.17 dans les deux sens, simulation) : aucun meneur.</t>
   </si>
   <si>
-    <t>Robusta sans la rupture de série du Vietnam (croissances 2012/13-2025/26, n = 14)</t>
+    <t>Robusta sans le saut de niveau du Vietnam (croissances 2012/13-2025/26, n = 14)</t>
   </si>
   <si>
     <t>DF (t−1) → production (t)</t>

</xml_diff>